<commit_message>
docs(tutorials): FEM-2 starter carries the LEM model only — every FEM input is entered on the page
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XjjT2aBxw8gY7EFdpoUcpj
</commit_message>
<xml_diff>
--- a/docs/tutorials/files/xslope_reinforced_slope_start.xlsx
+++ b/docs/tutorials/files/xslope_reinforced_slope_start.xlsx
@@ -6810,12 +6810,8 @@
         <v>0.0</v>
       </c>
       <c r="L11" s="3"/>
-      <c r="M11" s="3">
-        <v>1000000.0</v>
-      </c>
-      <c r="N11" s="3">
-        <v>0.3</v>
-      </c>
+      <c r="M11" s="3"/>
+      <c r="N11" s="3"/>
       <c r="O11" s="3" t="inlineStr">
         <is>
           <t>none</t>
@@ -6934,12 +6930,8 @@
         <v>0.0</v>
       </c>
       <c r="L12" s="3"/>
-      <c r="M12" s="3">
-        <v>1000000.0</v>
-      </c>
-      <c r="N12" s="3">
-        <v>0.3</v>
-      </c>
+      <c r="M12" s="3"/>
+      <c r="N12" s="3"/>
       <c r="O12" s="3" t="inlineStr">
         <is>
           <t>none</t>

</xml_diff>